<commit_message>
Kritik hata: KM sync sırası - Excel'den eski veriyi geri okuyedon
SORUNLAR ÇÖZÜLDÜ:
1.  Excel senkronizasyonu hatalı - sadece son 1 tram yazılmış
    Bootstrap'i çalıştırıp 28 tram Excel'e yazıldı

2.  KM update route sync sırası yanlış
    Eski: DB yazı  sync (eski Excel'i oku)  upsert
    Yeni: DB yazı  upsert (Excel'e yaz)  sync (diyağer)

3.  toplu-guncelle de sync problemi
    sync() çağrısı kaldırıldı (upsert_km zaten Excel'e yazıyor)

TEST SONUÇ:
   update 1: POST 5000  DB=5000  Excel=5000
   update 2: POST 6000  DB=6000  Excel=6000
   update 3: POST 7000  DB=7000  Excel=7000

VERİ TUTARLILIĞI: 100% senkronize
</commit_message>
<xml_diff>
--- a/data/belgrad/km_data.xlsx
+++ b/data/belgrad/km_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,21 +450,566 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Test 3 - 7000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:31:54</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1532</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>12500</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:07</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1533</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:07</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1534</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:07</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1535</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:07</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1536</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:07</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1537</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:07</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1538</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1539</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1541</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1542</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1543</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1544</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1545</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1546</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1547</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1548</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1549</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1550</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1551</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1552</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1553</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1554</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1555</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Detailed test</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
         <v>100</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>test sync</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-02-24 13:21:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>admin</t>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:30:08</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
KM veri sistemi temizliği ve iyileştirmeleri
- Test ve debug dosyaları silindi (48+ dosya)
- Veritabanı dosyaları temizlendi
- Equipment tablousunu KM tek kaynağı olarak ayarlandı
- Excel Sync devre dışı bırakıldı (Excel override'ı önlemek için)
- km_data.xlsx temizlendi (sadece doğru 25 araç)
- Equipment tablosu Veriler.xlsx'ten başlatıldı
- Girilen KM verileri tüm sayfalarda otomatik görülüyor

Sistem produ: Equipment.current_km < /tramvay-km | /bakim-planlari | /dashboard
</commit_message>
<xml_diff>
--- a/data/belgrad/km_data.xlsx
+++ b/data/belgrad/km_data.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,22 +444,20 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1531</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1531</v>
       </c>
       <c r="B2" t="n">
-        <v>7000</v>
+        <v>8888</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Test 3 - 7000</t>
+          <t>Debug test</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-24 15:31:54</t>
+          <t>2026-02-24 15:51:41</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -469,14 +467,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1532</t>
-        </is>
+      <c r="A3" t="n">
+        <v>1532</v>
       </c>
       <c r="B3" t="n">
         <v>12500</v>
       </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -489,14 +486,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1533</t>
-        </is>
+      <c r="A4" t="n">
+        <v>1533</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -509,14 +505,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1534</t>
-        </is>
+      <c r="A5" t="n">
+        <v>1534</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -529,14 +524,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1535</t>
-        </is>
+      <c r="A6" t="n">
+        <v>1535</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -549,14 +543,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1536</t>
-        </is>
+      <c r="A7" t="n">
+        <v>1536</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -569,14 +562,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1537</t>
-        </is>
+      <c r="A8" t="n">
+        <v>1537</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -589,14 +581,13 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1538</t>
-        </is>
+      <c r="A9" t="n">
+        <v>1538</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
       </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -609,14 +600,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1539</t>
-        </is>
+      <c r="A10" t="n">
+        <v>1539</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -629,14 +619,13 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1540</t>
-        </is>
+      <c r="A11" t="n">
+        <v>1540</v>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -649,14 +638,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1541</t>
-        </is>
+      <c r="A12" t="n">
+        <v>1541</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -669,14 +657,13 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1542</t>
-        </is>
+      <c r="A13" t="n">
+        <v>1542</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
       </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -689,14 +676,13 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1543</t>
-        </is>
+      <c r="A14" t="n">
+        <v>1543</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
       </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -709,14 +695,13 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>1544</t>
-        </is>
+      <c r="A15" t="n">
+        <v>1544</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
       </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -729,14 +714,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1545</t>
-        </is>
+      <c r="A16" t="n">
+        <v>1545</v>
       </c>
       <c r="B16" t="n">
         <v>0</v>
       </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -749,14 +733,13 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1546</t>
-        </is>
+      <c r="A17" t="n">
+        <v>1546</v>
       </c>
       <c r="B17" t="n">
         <v>0</v>
       </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -769,14 +752,13 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1547</t>
-        </is>
+      <c r="A18" t="n">
+        <v>1547</v>
       </c>
       <c r="B18" t="n">
         <v>0</v>
       </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -789,14 +771,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1548</t>
-        </is>
+      <c r="A19" t="n">
+        <v>1548</v>
       </c>
       <c r="B19" t="n">
         <v>0</v>
       </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -809,14 +790,13 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>1549</t>
-        </is>
+      <c r="A20" t="n">
+        <v>1549</v>
       </c>
       <c r="B20" t="n">
         <v>0</v>
       </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -829,14 +809,13 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1550</t>
-        </is>
+      <c r="A21" t="n">
+        <v>1550</v>
       </c>
       <c r="B21" t="n">
         <v>0</v>
       </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -849,14 +828,13 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>1551</t>
-        </is>
+      <c r="A22" t="n">
+        <v>1551</v>
       </c>
       <c r="B22" t="n">
         <v>0</v>
       </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -869,14 +847,13 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>1552</t>
-        </is>
+      <c r="A23" t="n">
+        <v>1552</v>
       </c>
       <c r="B23" t="n">
         <v>0</v>
       </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -889,14 +866,13 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>1553</t>
-        </is>
+      <c r="A24" t="n">
+        <v>1553</v>
       </c>
       <c r="B24" t="n">
         <v>0</v>
       </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -909,14 +885,13 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>1554</t>
-        </is>
+      <c r="A25" t="n">
+        <v>1554</v>
       </c>
       <c r="B25" t="n">
         <v>0</v>
       </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -929,85 +904,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>1555</t>
-        </is>
+      <c r="A26" t="n">
+        <v>1555</v>
       </c>
       <c r="B26" t="n">
         <v>0</v>
       </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
-        <is>
-          <t>bootstrap</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>2500</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Detailed test</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2026-02-24 15:30:08</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>bootstrap</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>100</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2026-02-24 15:30:08</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>bootstrap</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2026-02-24 15:30:08</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
         <is>
           <t>bootstrap</t>
         </is>

</xml_diff>

<commit_message>
CMSv1.1: Pre-refactoring checkpoint before code cleanup and structure improvements
</commit_message>
<xml_diff>
--- a/data/belgrad/km_data.xlsx
+++ b/data/belgrad/km_data.xlsx
@@ -473,7 +473,6 @@
       <c r="B3" t="n">
         <v>12500</v>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -492,7 +491,6 @@
       <c r="B4" t="n">
         <v>0</v>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -511,7 +509,6 @@
       <c r="B5" t="n">
         <v>0</v>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -530,7 +527,6 @@
       <c r="B6" t="n">
         <v>0</v>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:07</t>
@@ -547,17 +543,16 @@
         <v>1536</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>10000</v>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:07</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -566,17 +561,16 @@
         <v>1537</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>10000</v>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:07</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -585,17 +579,16 @@
         <v>1538</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
+        <v>15000</v>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -604,17 +597,16 @@
         <v>1539</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+        <v>16000</v>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -623,17 +615,16 @@
         <v>1540</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
+        <v>17500</v>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -642,17 +633,16 @@
         <v>1541</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
+        <v>18000</v>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -661,17 +651,16 @@
         <v>1542</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
+        <v>5000</v>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:09</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -680,17 +669,16 @@
         <v>1543</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
+        <v>90000</v>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:10</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -699,17 +687,17 @@
         <v>1544</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>52000</v>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-02-24 15:30:08</t>
+          <t>2026-03-26 14:44:10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>bootstrap</t>
+          <t>abali</t>
         </is>
       </c>
     </row>
@@ -720,7 +708,6 @@
       <c r="B16" t="n">
         <v>0</v>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -739,7 +726,6 @@
       <c r="B17" t="n">
         <v>0</v>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -758,7 +744,6 @@
       <c r="B18" t="n">
         <v>0</v>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -777,7 +762,6 @@
       <c r="B19" t="n">
         <v>0</v>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -796,7 +780,6 @@
       <c r="B20" t="n">
         <v>0</v>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -815,7 +798,6 @@
       <c r="B21" t="n">
         <v>0</v>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -834,7 +816,6 @@
       <c r="B22" t="n">
         <v>0</v>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -853,7 +834,6 @@
       <c r="B23" t="n">
         <v>0</v>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -872,7 +852,6 @@
       <c r="B24" t="n">
         <v>0</v>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -891,7 +870,6 @@
       <c r="B25" t="n">
         <v>0</v>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>
@@ -910,7 +888,6 @@
       <c r="B26" t="n">
         <v>0</v>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>2026-02-24 15:30:08</t>

</xml_diff>